<commit_message>
Add Phase Triggers tab to components spreadsheet
New tab documents trigger mode for all 8 phases:
- Automatic (🟢): RESTORE, INIT, BOOTSTRAP — fired by hooks, no user action needed
- Semi-automatic (🟣): CHECKPOINT, ONBOARD — hook reminds or escalates, user can also trigger manually
- Manual (🟠): START, QUICK-CHECK, END — user must state intent

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/claude-memory-guard-components.xlsx
+++ b/claude-memory-guard-components.xlsx
@@ -9,6 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hook Scripts" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Managed Files" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Triggers" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,8 +60,38 @@
       <family val="2"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -87,8 +118,38 @@
         <fgColor rgb="FFDCE6F1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00843C0C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007030A0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -170,11 +231,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="001F3864"/>
+      </left>
+      <right style="medium">
+        <color rgb="001F3864"/>
+      </right>
+      <top style="medium">
+        <color rgb="001F3864"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001F3864"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -202,6 +291,36 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -583,7 +702,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -638,7 +756,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
@@ -693,7 +810,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
@@ -1383,7 +1499,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
@@ -1449,7 +1564,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
@@ -1524,4 +1638,341 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" style="5" min="1" max="1"/>
+    <col width="18" customWidth="1" style="5" min="2" max="2"/>
+    <col width="28" customWidth="1" style="5" min="3" max="3"/>
+    <col width="52" customWidth="1" style="5" min="4" max="4"/>
+    <col width="38" customWidth="1" style="5" min="5" max="5"/>
+    <col width="36" customWidth="1" style="5" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1" s="5">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Phase Trigger Reference — claude-memory-guard</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1" s="5">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Trigger Mode:   🟢 Automatic — fired by a hook, no user action needed   🟣 Semi-automatic — hook fires a reminder, but Claude acts on it / user can also trigger manually   🟠 Manual — user must explicitly say the keyword or phrase</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" s="5">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>Trigger Mode</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>Triggered By</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>What Fires It</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>User Keywords</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>Hook Script Involved</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1" s="5">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>RESTORE</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>🟢 Automatic</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>SessionStart hook
+PostCompact hook</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>Fires on every new session start and after every /compact. Hook injects a mandatory reminder into Claude's context.</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>"continue", "resume"
+(optional — hook fires regardless)</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>session_start_reminder.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1" s="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>INIT</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>🟢 Automatic</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>SessionStart hook
+(condition: CLAUDE.md missing)</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>session_start_reminder.py detects missing CLAUDE.md and auto-creates it before Claude's first response. Agent phase then runs to confirm setup.</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>None required</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>session_start_reminder.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1" s="5">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>BOOTSTRAP</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>🟢 Automatic</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>SessionStart hook
+(condition: PROJECT_GUIDE.md missing)</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>session_start_reminder.py detects missing docs/PROJECT_GUIDE.md and auto-creates it. Agent phase runs to confirm and fill in structure.</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>None required</t>
+        </is>
+      </c>
+      <c r="F6" s="17" t="inlineStr">
+        <is>
+          <t>session_start_reminder.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1" s="5">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>START</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>🟠 Manual</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>User explicitly states a new coding goal or feature request in the conversation.</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>"I want to...", "add X", "fix Y", "build Z", "let's implement..."</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>None (Claude detects goal from conversation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1" s="5">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>QUICK-CHECK</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>🟠 Manual</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>User requests a small, targeted edit such as a typo fix, label change, or minor correction.</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>"fix this typo", "change X to Y", "rename this"</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>None (Claude detects small edit from conversation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1" s="5">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>CHECKPOINT</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>🟣 Semi-automatic</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>PostToolUse hook (every 10 tool calls)
+OR User</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>checkpoint_counter.py counts every tool call. At 10, it injects a CHECKPOINT reminder automatically. User can also trigger it manually at any time.</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>"checkpoint", "save state", "save progress"</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>checkpoint_counter.py
+checkpoint_memory.py (PreCompact safety net)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1" s="5">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>END</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>🟠 Manual</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>User signals that coding work is complete for the current task. Claude then runs END to update all documentation.</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>"done", "looks good", "we're done", "that's it"</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>end_reminder.py
+(reminds user to trigger END when task is active)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1" s="5">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>ONBOARD</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>🟣 Semi-automatic</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>User command
+OR RESTORE (condition: MEMORY.md missing on existing project)</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>User explicitly requests onboarding, OR RESTORE detects that MEMORY.md doesn't exist for a project that already has code — it then automatically escalates to ONBOARD.</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>"onboard this project", "set up claude-memory-guard"</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>session_start_reminder.py
+(RESTORE → ONBOARD escalation)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>